<commit_message>
Added dollar signs where missing
I went through each statement to restore formatting where it was missing.
</commit_message>
<xml_diff>
--- a/app/static/input_files/ACFR_template.xlsx
+++ b/app/static/input_files/ACFR_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sarrahahmed/Desktop/CLOSUP/process-xbrl/app/static/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7005A4-4327-964A-AA98-262F64B11467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93C9FE1-EF87-8943-A2C6-02B8CFDC486D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" tabRatio="834" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17280" tabRatio="834" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lookup Net Position" sheetId="8" r:id="rId1"/>
@@ -11697,7 +11697,7 @@
     <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="275">
+  <cellXfs count="270">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -12154,21 +12154,9 @@
     <xf numFmtId="165" fontId="23" fillId="13" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="10" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="10" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="165" fontId="1" fillId="10" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
@@ -12211,6 +12199,14 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="23" fillId="13" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="44" fontId="23" fillId="13" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -12243,14 +12239,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="44" fontId="23" fillId="13" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="44" fontId="23" fillId="13" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -20056,18 +20044,18 @@
       </c>
     </row>
     <row r="59" spans="1:10" ht="15">
-      <c r="A59" s="266" t="s">
+      <c r="A59" s="263" t="s">
         <v>3615</v>
       </c>
-      <c r="B59" s="267"/>
-      <c r="C59" s="267"/>
-      <c r="D59" s="267"/>
-      <c r="E59" s="267"/>
-      <c r="F59" s="267"/>
-      <c r="G59" s="267"/>
-      <c r="H59" s="267"/>
-      <c r="I59" s="267"/>
-      <c r="J59" s="268"/>
+      <c r="B59" s="264"/>
+      <c r="C59" s="264"/>
+      <c r="D59" s="264"/>
+      <c r="E59" s="264"/>
+      <c r="F59" s="264"/>
+      <c r="G59" s="264"/>
+      <c r="H59" s="264"/>
+      <c r="I59" s="264"/>
+      <c r="J59" s="265"/>
     </row>
     <row r="60" spans="1:10" ht="15">
       <c r="A60" s="108" t="str">
@@ -20082,7 +20070,7 @@
       <c r="G60" s="209"/>
       <c r="H60" s="210"/>
       <c r="I60" s="210"/>
-      <c r="J60" s="250">
+      <c r="J60" s="245">
         <v>0</v>
       </c>
     </row>
@@ -20099,23 +20087,23 @@
       <c r="G61" s="209"/>
       <c r="H61" s="210"/>
       <c r="I61" s="210"/>
-      <c r="J61" s="250">
+      <c r="J61" s="245">
         <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="15">
-      <c r="A62" s="266" t="s">
+      <c r="A62" s="263" t="s">
         <v>3616</v>
       </c>
-      <c r="B62" s="267"/>
-      <c r="C62" s="267"/>
-      <c r="D62" s="267"/>
-      <c r="E62" s="267"/>
-      <c r="F62" s="267"/>
-      <c r="G62" s="267"/>
-      <c r="H62" s="267"/>
-      <c r="I62" s="267"/>
-      <c r="J62" s="268"/>
+      <c r="B62" s="264"/>
+      <c r="C62" s="264"/>
+      <c r="D62" s="264"/>
+      <c r="E62" s="264"/>
+      <c r="F62" s="264"/>
+      <c r="G62" s="264"/>
+      <c r="H62" s="264"/>
+      <c r="I62" s="264"/>
+      <c r="J62" s="265"/>
     </row>
     <row r="63" spans="1:10" ht="15">
       <c r="A63" s="108" t="str">
@@ -20130,7 +20118,7 @@
       <c r="G63" s="209"/>
       <c r="H63" s="210"/>
       <c r="I63" s="210"/>
-      <c r="J63" s="249">
+      <c r="J63" s="244">
         <v>0</v>
       </c>
     </row>
@@ -20147,23 +20135,23 @@
       <c r="G64" s="209"/>
       <c r="H64" s="210"/>
       <c r="I64" s="210"/>
-      <c r="J64" s="249">
+      <c r="J64" s="244">
         <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="15">
-      <c r="A65" s="266" t="s">
+      <c r="A65" s="263" t="s">
         <v>3617</v>
       </c>
-      <c r="B65" s="267"/>
-      <c r="C65" s="267"/>
-      <c r="D65" s="267"/>
-      <c r="E65" s="267"/>
-      <c r="F65" s="267"/>
-      <c r="G65" s="267"/>
-      <c r="H65" s="267"/>
-      <c r="I65" s="267"/>
-      <c r="J65" s="268"/>
+      <c r="B65" s="264"/>
+      <c r="C65" s="264"/>
+      <c r="D65" s="264"/>
+      <c r="E65" s="264"/>
+      <c r="F65" s="264"/>
+      <c r="G65" s="264"/>
+      <c r="H65" s="264"/>
+      <c r="I65" s="264"/>
+      <c r="J65" s="265"/>
     </row>
     <row r="66" spans="1:10" ht="16">
       <c r="A66" s="131" t="str">
@@ -20178,7 +20166,7 @@
       <c r="G66" s="209"/>
       <c r="H66" s="210"/>
       <c r="I66" s="210"/>
-      <c r="J66" s="249">
+      <c r="J66" s="244">
         <v>0</v>
       </c>
     </row>
@@ -20195,7 +20183,7 @@
       <c r="G67" s="209"/>
       <c r="H67" s="210"/>
       <c r="I67" s="210"/>
-      <c r="J67" s="249">
+      <c r="J67" s="244">
         <v>0</v>
       </c>
     </row>
@@ -20258,7 +20246,10 @@
         <f>SUM(E68, E45, E32)</f>
         <v>0</v>
       </c>
-      <c r="F69" s="219"/>
+      <c r="F69" s="219">
+        <f>SUM(F68, F45, F32)</f>
+        <v>0</v>
+      </c>
       <c r="G69" s="219">
         <f>SUM(G68, G45, G32)</f>
         <v>0</v>
@@ -20277,14 +20268,14 @@
       </c>
     </row>
     <row r="72" spans="1:10">
-      <c r="A72" s="258"/>
-      <c r="B72" s="264" t="s">
+      <c r="A72" s="253"/>
+      <c r="B72" s="261" t="s">
         <v>3636</v>
       </c>
     </row>
     <row r="73" spans="1:10">
-      <c r="A73" s="258"/>
-      <c r="B73" s="265"/>
+      <c r="A73" s="253"/>
+      <c r="B73" s="262"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -20444,7 +20435,7 @@
         <v>44742</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="32">
+    <row r="6" spans="1:2" ht="16">
       <c r="A6" s="173" t="s">
         <v>2465</v>
       </c>
@@ -20481,7 +20472,7 @@
       <c r="B13" s="210"/>
     </row>
     <row r="14" spans="1:2" ht="15">
-      <c r="A14" s="273" t="s">
+      <c r="A14" s="257" t="s">
         <v>3638</v>
       </c>
       <c r="B14" s="210">
@@ -20512,7 +20503,7 @@
       <c r="B19" s="210"/>
     </row>
     <row r="20" spans="1:2" ht="15">
-      <c r="A20" s="273" t="s">
+      <c r="A20" s="257" t="s">
         <v>3639</v>
       </c>
       <c r="B20" s="210">
@@ -20543,7 +20534,7 @@
       <c r="B25" s="210"/>
     </row>
     <row r="26" spans="1:2" ht="15">
-      <c r="A26" s="274" t="s">
+      <c r="A26" s="258" t="s">
         <v>3640</v>
       </c>
       <c r="B26" s="210">
@@ -20574,7 +20565,7 @@
       <c r="B31" s="210"/>
     </row>
     <row r="32" spans="1:2" ht="15">
-      <c r="A32" s="273" t="s">
+      <c r="A32" s="257" t="s">
         <v>3641</v>
       </c>
       <c r="B32" s="224">
@@ -20592,14 +20583,14 @@
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="269" t="s">
+      <c r="A36" s="266" t="s">
         <v>3636</v>
       </c>
-      <c r="B36" s="264"/>
+      <c r="B36" s="261"/>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="270"/>
-      <c r="B37" s="265"/>
+      <c r="A37" s="267"/>
+      <c r="B37" s="262"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -21972,14 +21963,14 @@
       <c r="J71" s="20"/>
     </row>
     <row r="72" spans="1:10">
-      <c r="A72" s="255"/>
-      <c r="B72" s="253" t="s">
+      <c r="A72" s="250"/>
+      <c r="B72" s="248" t="s">
         <v>3636</v>
       </c>
     </row>
     <row r="73" spans="1:10">
-      <c r="A73" s="255"/>
-      <c r="B73" s="254"/>
+      <c r="A73" s="250"/>
+      <c r="B73" s="249"/>
     </row>
   </sheetData>
   <sheetProtection formatRows="0" insertRows="0" deleteRows="0"/>
@@ -22130,7 +22121,7 @@
       <c r="B12" s="210"/>
     </row>
     <row r="13" spans="1:2" ht="15">
-      <c r="A13" s="273" t="s">
+      <c r="A13" s="257" t="s">
         <v>3642</v>
       </c>
       <c r="B13" s="210">
@@ -22161,7 +22152,7 @@
       <c r="B18" s="210"/>
     </row>
     <row r="19" spans="1:2" ht="15">
-      <c r="A19" s="273" t="s">
+      <c r="A19" s="257" t="s">
         <v>3643</v>
       </c>
       <c r="B19" s="210">
@@ -22192,7 +22183,7 @@
       <c r="B24" s="210"/>
     </row>
     <row r="25" spans="1:2" ht="15">
-      <c r="A25" s="273" t="s">
+      <c r="A25" s="257" t="s">
         <v>3644</v>
       </c>
       <c r="B25" s="210">
@@ -22207,14 +22198,14 @@
       <c r="B26" s="175"/>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="269" t="s">
+      <c r="A29" s="266" t="s">
         <v>3636</v>
       </c>
-      <c r="B29" s="264"/>
+      <c r="B29" s="261"/>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="270"/>
-      <c r="B30" s="265"/>
+      <c r="A30" s="267"/>
+      <c r="B30" s="262"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -22655,29 +22646,29 @@
         <f>SUM(C10:C23)</f>
         <v>0</v>
       </c>
-      <c r="D24" s="231" t="str">
-        <f t="shared" ref="D24:I24" si="1">IF(D$7="Type fund name","",SUM(D10:D23))</f>
-        <v/>
-      </c>
-      <c r="E24" s="231" t="str">
+      <c r="D24" s="231">
+        <f t="shared" ref="D24:I24" si="1">SUM(D10:D23)</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="F24" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F24" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G24" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G24" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H24" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H24" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I24" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I24" s="231">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J24" s="231">
         <f>IF(J7="","",SUM(J10:J23))</f>
@@ -22925,29 +22916,29 @@
         <f>SUM(C26:C32)</f>
         <v>0</v>
       </c>
-      <c r="D38" s="231" t="str">
-        <f t="shared" ref="D38:I38" si="4">IF(D$7="Type fund name","",SUM(D26:D32))</f>
-        <v/>
-      </c>
-      <c r="E38" s="231" t="str">
+      <c r="D38" s="231">
+        <f t="shared" ref="D38:I38" si="4">SUM(D26:D32)</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="231">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="F38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F38" s="231">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="G38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G38" s="231">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H38" s="231">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I38" s="231">
         <f t="shared" si="4"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J38" s="231">
         <f>IF(J7="","",SUM(J26:J37))</f>
@@ -22965,29 +22956,29 @@
         <f>C24+C38</f>
         <v>0</v>
       </c>
-      <c r="D39" s="232" t="str">
-        <f t="shared" ref="D39:I39" si="5">IF(D$7="Type fund name","",D24+D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="232" t="str">
+      <c r="D39" s="219">
+        <f t="shared" ref="D39:I39" si="5">D24+D38</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="219">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="F39" s="232" t="str">
+        <v>0</v>
+      </c>
+      <c r="F39" s="219">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="G39" s="232" t="str">
+        <v>0</v>
+      </c>
+      <c r="G39" s="219">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="H39" s="232" t="str">
+        <v>0</v>
+      </c>
+      <c r="H39" s="219">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="I39" s="232" t="str">
+        <v>0</v>
+      </c>
+      <c r="I39" s="219">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J39" s="219">
         <f>IF(J7="","",J24+J38)</f>
@@ -23229,29 +23220,29 @@
         <f>IF(C$7="","",SUM(C42:C52))</f>
         <v>0</v>
       </c>
-      <c r="D53" s="231" t="str">
-        <f t="shared" ref="D53:I53" si="7">IF(D$7="Type fund name","",SUM(D42:D52))</f>
-        <v/>
-      </c>
-      <c r="E53" s="231" t="str">
+      <c r="D53" s="231">
+        <f t="shared" ref="D53:I53" si="7">IF(D$7="","",SUM(D42:D52))</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="231">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="F53" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F53" s="231">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="G53" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G53" s="231">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H53" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H53" s="231">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="I53" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I53" s="231">
         <f t="shared" si="7"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J53" s="231">
         <f t="shared" si="6"/>
@@ -23507,29 +23498,29 @@
         <f>IF(C$7="","",SUM(C57:C67))</f>
         <v>0</v>
       </c>
-      <c r="D68" s="231" t="str">
-        <f t="shared" ref="D68:I68" si="10">IF(D$7="Type fund name","",SUM(D57:D67))</f>
-        <v/>
-      </c>
-      <c r="E68" s="231" t="str">
+      <c r="D68" s="231">
+        <f t="shared" ref="D68:I68" si="10">IF(D$7="","",SUM(D57:D67))</f>
+        <v>0</v>
+      </c>
+      <c r="E68" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F68" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F68" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="G68" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G68" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="H68" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H68" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="I68" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I68" s="231">
         <f t="shared" si="10"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J68" s="231">
         <f t="shared" si="8"/>
@@ -23768,29 +23759,29 @@
         <f>SUM(C70:C78)</f>
         <v>0</v>
       </c>
-      <c r="D82" s="231" t="str">
-        <f t="shared" ref="D82:I82" si="13">IF(D$7="Type fund name","",SUM(D70:D78))</f>
-        <v/>
-      </c>
-      <c r="E82" s="231" t="str">
+      <c r="D82" s="231">
+        <f t="shared" ref="D82:I82" si="13">SUM(D70:D78)</f>
+        <v>0</v>
+      </c>
+      <c r="E82" s="231">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="F82" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F82" s="231">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="G82" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G82" s="231">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="H82" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H82" s="231">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="I82" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I82" s="231">
         <f t="shared" si="13"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J82" s="231">
         <f t="shared" si="11"/>
@@ -23808,29 +23799,29 @@
         <f>C68+C82</f>
         <v>0</v>
       </c>
-      <c r="D83" s="219" t="str">
-        <f t="shared" ref="D83:I83" si="14">IF(D$7 = "Type fund name", "", D68+D82)</f>
-        <v/>
-      </c>
-      <c r="E83" s="219" t="str">
+      <c r="D83" s="219">
+        <f t="shared" ref="D83:I83" si="14">D68+D82</f>
+        <v>0</v>
+      </c>
+      <c r="E83" s="219">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="F83" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="F83" s="219">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="G83" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="G83" s="219">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="H83" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="H83" s="219">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="I83" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="I83" s="219">
         <f t="shared" si="14"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J83" s="233">
         <f t="shared" si="11"/>
@@ -24072,29 +24063,29 @@
         <f>IF(C$7="","",SUM(C86:C96))</f>
         <v>0</v>
       </c>
-      <c r="D97" s="231" t="str">
-        <f t="shared" ref="D97:I97" si="16">IF(D$7="Type fund name","",SUM(D86:D96))</f>
-        <v/>
-      </c>
-      <c r="E97" s="231" t="str">
+      <c r="D97" s="231">
+        <f t="shared" ref="D97:I97" si="16">IF(D$7="","",SUM(D86:D96))</f>
+        <v>0</v>
+      </c>
+      <c r="E97" s="231">
         <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="F97" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F97" s="231">
         <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="G97" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G97" s="231">
         <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="H97" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H97" s="231">
         <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="I97" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I97" s="231">
         <f t="shared" si="16"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J97" s="231">
         <f t="shared" si="15"/>
@@ -24300,29 +24291,29 @@
         <f>IF(C7="","",SUM(C100:C108))</f>
         <v>0</v>
       </c>
-      <c r="D109" s="219" t="str">
-        <f t="shared" ref="D109:I109" si="18">IF(D7="Type fund name","",SUM(D100:D108))</f>
-        <v/>
-      </c>
-      <c r="E109" s="219" t="str">
+      <c r="D109" s="219">
+        <f t="shared" ref="D109:I109" si="18">IF(D7="","",SUM(D100:D108))</f>
+        <v>0</v>
+      </c>
+      <c r="E109" s="219">
         <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="F109" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="F109" s="219">
         <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="G109" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="G109" s="219">
         <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="H109" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="H109" s="219">
         <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="I109" s="219" t="str">
+        <v>0</v>
+      </c>
+      <c r="I109" s="219">
         <f t="shared" si="18"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J109" s="232">
         <f t="shared" si="17"/>
@@ -24354,8 +24345,8 @@
       <c r="J111" s="112"/>
     </row>
     <row r="112" spans="1:10" s="33" customFormat="1" ht="15" hidden="1">
-      <c r="A112" s="257"/>
-      <c r="B112" s="262" t="s">
+      <c r="A112" s="252"/>
+      <c r="B112" s="259" t="s">
         <v>3636</v>
       </c>
       <c r="C112" s="84"/>
@@ -24368,8 +24359,8 @@
       <c r="J112" s="112"/>
     </row>
     <row r="113" spans="1:10" s="33" customFormat="1" ht="15" hidden="1">
-      <c r="A113" s="257"/>
-      <c r="B113" s="263"/>
+      <c r="A113" s="252"/>
+      <c r="B113" s="260"/>
       <c r="C113" s="84"/>
       <c r="D113" s="84"/>
       <c r="E113" s="84"/>
@@ -24443,7 +24434,7 @@
       <formula>NOT(ISERROR(SEARCH("custom",A100)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C24 C38 C68:I68 C82:C83 C109:I109">
+  <conditionalFormatting sqref="C24:I24 C38:I38 C68:I68 C82:I83 C109:I109">
     <cfRule type="expression" dxfId="40" priority="20" stopIfTrue="1">
       <formula>C$7=""</formula>
     </cfRule>
@@ -24456,11 +24447,6 @@
   <conditionalFormatting sqref="C97:I97">
     <cfRule type="expression" dxfId="38" priority="2" stopIfTrue="1">
       <formula>C$7=""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D82:I82">
-    <cfRule type="expression" dxfId="37" priority="18" stopIfTrue="1">
-      <formula>D$7=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7">
@@ -24937,29 +24923,29 @@
         <f>IF(C$7="","",SUM(C9:C22))</f>
         <v>0</v>
       </c>
-      <c r="D23" s="231" t="str">
-        <f t="shared" ref="D23:I23" si="1">IF(D$7="Type fund name","",SUM(D9:D22))</f>
-        <v/>
-      </c>
-      <c r="E23" s="231" t="str">
+      <c r="D23" s="231">
+        <f t="shared" ref="D23:I23" si="1">IF(D$7="","",SUM(D9:D22))</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="F23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I23" s="231">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J23" s="231">
         <f>IF(J7="","",SUM(J9:J22))</f>
@@ -25219,29 +25205,29 @@
         <f>IF(C7="","",SUM(C26:C32))</f>
         <v>0</v>
       </c>
-      <c r="D38" s="231" t="str">
-        <f t="shared" ref="D38:I38" si="3">IF(D$7="Type fund name","",SUM(D26:D32))</f>
-        <v/>
-      </c>
-      <c r="E38" s="231" t="str">
+      <c r="D38" s="231">
+        <f t="shared" ref="D38:I38" si="3">IF(D7="","",SUM(D26:D32))</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="231">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="F38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F38" s="231">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G38" s="231">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="H38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H38" s="231">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I38" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I38" s="231">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J38" s="231">
         <f>IF(J7="","",SUM(J26:J37))</f>
@@ -25480,29 +25466,29 @@
         <f>IF(C7="","",SUM(C41:C51))</f>
         <v>0</v>
       </c>
-      <c r="D52" s="231" t="str">
-        <f t="shared" ref="D52:I52" si="6">IF(D$7="Type fund name","",SUM(D41:D51))</f>
-        <v/>
-      </c>
-      <c r="E52" s="231" t="str">
+      <c r="D52" s="231">
+        <f t="shared" ref="D52:I52" si="6">IF(D7="","",SUM(D41:D51))</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="231">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="F52" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F52" s="231">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="G52" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G52" s="231">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H52" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H52" s="231">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="I52" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I52" s="231">
         <f t="shared" si="6"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J52" s="231">
         <f t="shared" si="4"/>
@@ -25521,11 +25507,11 @@
         <v>0</v>
       </c>
       <c r="D53" s="232" t="str">
-        <f t="shared" ref="D53:I53" si="7">IF(D$7="Type fund name","",D23-D38+D52)</f>
+        <f>IF(D$7="Type fund name","",D23-D38+D52)</f>
         <v/>
       </c>
       <c r="E53" s="232" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="D53:I53" si="7">IF(E$7="Type fund name","",E23-E38+E52)</f>
         <v/>
       </c>
       <c r="F53" s="232" t="str">
@@ -25748,29 +25734,29 @@
         <f>IF(C7="","",SUM(C56:C64))</f>
         <v>0</v>
       </c>
-      <c r="D65" s="231" t="str">
-        <f t="shared" ref="D65:I65" si="10">IF(D$7="Type fund name","",SUM(D56:D64))</f>
-        <v/>
-      </c>
-      <c r="E65" s="231" t="str">
+      <c r="D65" s="231">
+        <f t="shared" ref="D65:I65" si="10">IF(D7="","",SUM(D56:D64))</f>
+        <v>0</v>
+      </c>
+      <c r="E65" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="F65" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F65" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="G65" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G65" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="H65" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H65" s="231">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="I65" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I65" s="231">
         <f t="shared" si="10"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J65" s="231">
         <f t="shared" si="8"/>
@@ -25789,10 +25775,13 @@
         <v>0</v>
       </c>
       <c r="D66" s="233" t="str">
-        <f t="shared" ref="D66:I66" si="11">IF(D$7="Type fund name","",D53+D65)</f>
+        <f>IF(D$7="Type fund name","",D53+D65)</f>
         <v/>
       </c>
-      <c r="E66" s="233"/>
+      <c r="E66" s="233" t="str">
+        <f t="shared" ref="D66:I66" si="11">IF(E$7="Type fund name","",E53+E65)</f>
+        <v/>
+      </c>
       <c r="F66" s="233" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -25913,15 +25902,15 @@
       <c r="J72" s="112"/>
     </row>
     <row r="73" spans="1:10" ht="15">
-      <c r="A73" s="259"/>
-      <c r="B73" s="271" t="s">
+      <c r="A73" s="254"/>
+      <c r="B73" s="268" t="s">
         <v>3636</v>
       </c>
       <c r="J73" s="112"/>
     </row>
     <row r="74" spans="1:10" ht="15">
-      <c r="A74" s="259"/>
-      <c r="B74" s="272"/>
+      <c r="A74" s="254"/>
+      <c r="B74" s="269"/>
       <c r="J74" s="112"/>
     </row>
     <row r="75" spans="1:10" ht="15">
@@ -26024,7 +26013,7 @@
       <formula>NOT(ISERROR(SEARCH("custom",A56)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C23:C24 C38:C39 C70:J70">
+  <conditionalFormatting sqref="C23:C24 C38:C39 C70:J70 D23:I23 D38:I38">
     <cfRule type="expression" dxfId="31" priority="15" stopIfTrue="1">
       <formula>C$7=""</formula>
     </cfRule>
@@ -26500,32 +26489,32 @@
         <f>IF(C$7="","",SUM(C9:C22))</f>
         <v>0</v>
       </c>
-      <c r="D23" s="231" t="str">
-        <f t="shared" ref="D23:J23" si="1">IF(D$7="Type fund name","",SUM(D9:D22))</f>
-        <v/>
-      </c>
-      <c r="E23" s="231" t="str">
+      <c r="D23" s="231">
+        <f t="shared" ref="D23:I23" si="1">IF(D$7="","",SUM(D9:D22))</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="F23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="F23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="G23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="H23" s="231">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I23" s="231" t="str">
+        <v>0</v>
+      </c>
+      <c r="I23" s="231">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J23" s="231">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="J23" si="2">IF(J$7="Type fund name","",SUM(J9:J22))</f>
         <v>0</v>
       </c>
     </row>
@@ -26589,7 +26578,7 @@
       <c r="H27" s="208"/>
       <c r="I27" s="208"/>
       <c r="J27" s="235">
-        <f t="shared" ref="J27:J38" si="2">SUM(D27:I27)</f>
+        <f t="shared" ref="J27:J38" si="3">SUM(D27:I27)</f>
         <v>0</v>
       </c>
     </row>
@@ -26608,7 +26597,7 @@
       <c r="H28" s="208"/>
       <c r="I28" s="208"/>
       <c r="J28" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26627,7 +26616,7 @@
       <c r="H29" s="208"/>
       <c r="I29" s="208"/>
       <c r="J29" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26646,7 +26635,7 @@
       <c r="H30" s="208"/>
       <c r="I30" s="208"/>
       <c r="J30" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26665,7 +26654,7 @@
       <c r="H31" s="208"/>
       <c r="I31" s="208"/>
       <c r="J31" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26684,7 +26673,7 @@
       <c r="H32" s="208"/>
       <c r="I32" s="208"/>
       <c r="J32" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26703,7 +26692,7 @@
       <c r="H33" s="208"/>
       <c r="I33" s="208"/>
       <c r="J33" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26722,7 +26711,7 @@
       <c r="H34" s="208"/>
       <c r="I34" s="208"/>
       <c r="J34" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26741,7 +26730,7 @@
       <c r="H35" s="208"/>
       <c r="I35" s="208"/>
       <c r="J35" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26760,7 +26749,7 @@
       <c r="H36" s="208"/>
       <c r="I36" s="208"/>
       <c r="J36" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26779,7 +26768,7 @@
       <c r="H37" s="208"/>
       <c r="I37" s="208"/>
       <c r="J37" s="235">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -26794,32 +26783,32 @@
         <f>IF(C7="","",SUM(C26:C37))</f>
         <v>0</v>
       </c>
-      <c r="D38" s="231" t="str">
-        <f t="shared" ref="D38:I38" si="3">IF(D$7="Type fund name","",SUM(D26:D32))</f>
-        <v/>
-      </c>
-      <c r="E38" s="231" t="str">
+      <c r="D38" s="200">
+        <f t="shared" ref="D38:I38" si="4">IF(D7="","",SUM(D26:D37))</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="200">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F38" s="200">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G38" s="200">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="H38" s="200">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I38" s="200">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J38" s="235">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="F38" s="231" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G38" s="231" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="H38" s="231" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I38" s="231" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J38" s="235">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -26883,7 +26872,7 @@
       <c r="H42" s="209"/>
       <c r="I42" s="209"/>
       <c r="J42" s="235">
-        <f t="shared" ref="J42:J64" si="4">SUM(D42:I42)</f>
+        <f t="shared" ref="J42:J64" si="5">SUM(D42:I42)</f>
         <v>0</v>
       </c>
     </row>
@@ -26902,7 +26891,7 @@
       <c r="H43" s="208"/>
       <c r="I43" s="208"/>
       <c r="J43" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26921,7 +26910,7 @@
       <c r="H44" s="208"/>
       <c r="I44" s="208"/>
       <c r="J44" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26940,7 +26929,7 @@
       <c r="H45" s="208"/>
       <c r="I45" s="208"/>
       <c r="J45" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26959,7 +26948,7 @@
       <c r="H46" s="208"/>
       <c r="I46" s="208"/>
       <c r="J46" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26978,7 +26967,7 @@
       <c r="H47" s="208"/>
       <c r="I47" s="208"/>
       <c r="J47" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -26997,7 +26986,7 @@
       <c r="H48" s="208"/>
       <c r="I48" s="208"/>
       <c r="J48" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27016,7 +27005,7 @@
       <c r="H49" s="208"/>
       <c r="I49" s="208"/>
       <c r="J49" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27035,7 +27024,7 @@
       <c r="H50" s="208"/>
       <c r="I50" s="208"/>
       <c r="J50" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27054,7 +27043,7 @@
       <c r="H51" s="208"/>
       <c r="I51" s="208"/>
       <c r="J51" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27069,32 +27058,32 @@
         <f>IF(C7="","",SUM(C41:C51))</f>
         <v>0</v>
       </c>
-      <c r="D52" s="231" t="str">
-        <f t="shared" ref="D52:I52" si="5">IF(D$7="Type fund name","",SUM(D41:D51))</f>
-        <v/>
-      </c>
-      <c r="E52" s="231" t="str">
+      <c r="D52" s="200">
+        <f t="shared" ref="D52:I52" si="6">IF(D7="","",SUM(D41:D51))</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="200">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F52" s="200">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="G52" s="200">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H52" s="200">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="I52" s="200">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J52" s="235">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="F52" s="231" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="G52" s="231" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="H52" s="231" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="I52" s="231" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="J52" s="235">
-        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -27139,7 +27128,7 @@
       <c r="H55" s="208"/>
       <c r="I55" s="208"/>
       <c r="J55" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27158,7 +27147,7 @@
       <c r="H56" s="208"/>
       <c r="I56" s="208"/>
       <c r="J56" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27177,7 +27166,7 @@
       <c r="H57" s="208"/>
       <c r="I57" s="208"/>
       <c r="J57" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27196,7 +27185,7 @@
       <c r="H58" s="208"/>
       <c r="I58" s="208"/>
       <c r="J58" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27215,7 +27204,7 @@
       <c r="H59" s="208"/>
       <c r="I59" s="208"/>
       <c r="J59" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27234,7 +27223,7 @@
       <c r="H60" s="208"/>
       <c r="I60" s="208"/>
       <c r="J60" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27253,7 +27242,7 @@
       <c r="H61" s="208"/>
       <c r="I61" s="208"/>
       <c r="J61" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27272,7 +27261,7 @@
       <c r="H62" s="208"/>
       <c r="I62" s="208"/>
       <c r="J62" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27291,7 +27280,7 @@
       <c r="H63" s="208"/>
       <c r="I63" s="208"/>
       <c r="J63" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27306,32 +27295,32 @@
         <f>IF(C7="","",SUM(C55:C63))</f>
         <v>0</v>
       </c>
-      <c r="D64" s="231" t="str">
-        <f t="shared" ref="D64:I64" si="6">IF(D$7="Type fund name","",SUM(D55:D63))</f>
-        <v/>
-      </c>
-      <c r="E64" s="231" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="F64" s="231" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="G64" s="231" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H64" s="231" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="I64" s="231" t="str">
-        <f t="shared" si="6"/>
-        <v/>
+      <c r="D64" s="231">
+        <f t="shared" ref="D64:H64" si="7">IF(D7="","",SUM(D55:D63))</f>
+        <v>0</v>
+      </c>
+      <c r="E64" s="231">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F64" s="231">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="G64" s="231">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="H64" s="231">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="I64" s="231">
+        <f>IF(I7="","",SUM(I55:I63))</f>
+        <v>0</v>
       </c>
       <c r="J64" s="235">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -27346,32 +27335,32 @@
         <f>C23+C38+C52+C64</f>
         <v>0</v>
       </c>
-      <c r="D65" s="219" t="str">
-        <f t="shared" ref="D65:J65" si="7">IF(D7="Type fund name","",D23+D38+D52+D64)</f>
-        <v/>
-      </c>
-      <c r="E65" s="219" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="F65" s="219" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="G65" s="219" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H65" s="219" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="I65" s="219" t="str">
-        <f t="shared" si="7"/>
-        <v/>
+      <c r="D65" s="236">
+        <f t="shared" ref="D65:I65" si="8">D23+D38+D52+D64</f>
+        <v>0</v>
+      </c>
+      <c r="E65" s="236">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F65" s="236">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G65" s="236">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="H65" s="236">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I65" s="236">
+        <f t="shared" si="8"/>
+        <v>0</v>
       </c>
       <c r="J65" s="219">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="J65" si="9">IF(J7="Type fund name","",J23+J38+J52+J64)</f>
         <v>0</v>
       </c>
     </row>
@@ -27416,7 +27405,7 @@
       <c r="H68" s="237"/>
       <c r="I68" s="237"/>
       <c r="J68" s="235">
-        <f t="shared" ref="J68" si="8">SUM(D68:I68)</f>
+        <f t="shared" ref="J68" si="10">SUM(D68:I68)</f>
         <v>0</v>
       </c>
     </row>
@@ -27427,29 +27416,32 @@
       <c r="B69" s="152" t="s">
         <v>2463</v>
       </c>
-      <c r="C69" s="238"/>
+      <c r="C69" s="219">
+        <f>IF(C7="Type fund name","",C65+C68)</f>
+        <v>0</v>
+      </c>
       <c r="D69" s="219" t="str">
-        <f t="shared" ref="D69:I69" si="9">IF(D7="Type fund name","",D65+D68)</f>
+        <f>IF(D7="Type fund name","",D65+D68)</f>
         <v/>
       </c>
       <c r="E69" s="219" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="D69:I69" si="11">IF(E7="Type fund name","",E65+E68)</f>
         <v/>
       </c>
       <c r="F69" s="219" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G69" s="219" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="H69" s="219" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="I69" s="219" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="J69" s="219">
@@ -27542,8 +27534,8 @@
       <c r="J76" s="138"/>
     </row>
     <row r="77" spans="1:10" ht="15">
-      <c r="A77" s="257"/>
-      <c r="B77" s="262" t="s">
+      <c r="A77" s="252"/>
+      <c r="B77" s="259" t="s">
         <v>3636</v>
       </c>
       <c r="C77" s="155"/>
@@ -27556,8 +27548,8 @@
       <c r="J77" s="138"/>
     </row>
     <row r="78" spans="1:10" ht="15">
-      <c r="A78" s="257"/>
-      <c r="B78" s="263"/>
+      <c r="A78" s="252"/>
+      <c r="B78" s="260"/>
       <c r="C78" s="155"/>
       <c r="D78" s="155"/>
       <c r="E78" s="155"/>
@@ -27602,12 +27594,12 @@
       <formula>NOT(ISERROR(SEARCH("custom",A55)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
+  <conditionalFormatting sqref="C23:I23">
     <cfRule type="expression" dxfId="19" priority="22" stopIfTrue="1">
       <formula>C$7=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C38">
+  <conditionalFormatting sqref="C38:I38">
     <cfRule type="expression" dxfId="18" priority="21" stopIfTrue="1">
       <formula>C$7=""</formula>
     </cfRule>
@@ -27627,14 +27619,14 @@
       <formula>C$7=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D69:I69">
+  <conditionalFormatting sqref="C69:I69">
     <cfRule type="expression" dxfId="14" priority="16" stopIfTrue="1">
       <formula>#REF!=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D65:J65">
+  <conditionalFormatting sqref="J65">
     <cfRule type="expression" dxfId="13" priority="7" stopIfTrue="1">
-      <formula>D$7=""</formula>
+      <formula>J$7=""</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="12" priority="8" stopIfTrue="1" operator="equal">
       <formula>0</formula>
@@ -27649,9 +27641,9 @@
       <formula>#REF!=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D69:J69">
+  <conditionalFormatting sqref="C69:J69">
     <cfRule type="expression" dxfId="8" priority="12" stopIfTrue="1">
-      <formula>D$7=""</formula>
+      <formula>C$7=""</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="13" stopIfTrue="1" operator="equal">
       <formula>0</formula>
@@ -30939,7 +30931,7 @@
       <c r="C340" s="184"/>
     </row>
     <row r="341" spans="3:3" ht="15">
-      <c r="C341" s="241"/>
+      <c r="C341" s="240"/>
     </row>
     <row r="342" spans="3:3" ht="15">
       <c r="C342" s="184"/>
@@ -41017,19 +41009,19 @@
       <c r="C121" s="184"/>
     </row>
     <row r="122" spans="3:3" ht="15">
-      <c r="C122" s="239"/>
+      <c r="C122" s="238"/>
     </row>
     <row r="123" spans="3:3" ht="15">
-      <c r="C123" s="239"/>
+      <c r="C123" s="238"/>
     </row>
     <row r="124" spans="3:3" ht="15">
-      <c r="C124" s="239"/>
+      <c r="C124" s="238"/>
     </row>
     <row r="125" spans="3:3" ht="15">
-      <c r="C125" s="239"/>
+      <c r="C125" s="238"/>
     </row>
     <row r="126" spans="3:3" ht="15">
-      <c r="C126" s="240"/>
+      <c r="C126" s="239"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D126">
@@ -47363,7 +47355,7 @@
       <c r="C413" s="21"/>
     </row>
     <row r="414" spans="3:3" ht="15">
-      <c r="C414" s="248"/>
+      <c r="C414" s="243"/>
     </row>
     <row r="415" spans="3:3" ht="15">
       <c r="C415" s="21"/>
@@ -47512,7 +47504,7 @@
       <c r="E6" s="2"/>
     </row>
     <row r="10" spans="2:5" ht="14">
-      <c r="B10" s="252" t="s">
+      <c r="B10" s="247" t="s">
         <v>3634</v>
       </c>
     </row>
@@ -47587,7 +47579,7 @@
       </c>
     </row>
     <row r="29" spans="2:2">
-      <c r="B29" s="261" t="s">
+      <c r="B29" s="256" t="s">
         <v>3637</v>
       </c>
     </row>
@@ -47607,7 +47599,7 @@
       </c>
     </row>
     <row r="40" spans="2:2">
-      <c r="B40" s="260"/>
+      <c r="B40" s="255"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -47821,7 +47813,7 @@
         <f>IF(B16="","Choose from drop-down --&gt;",IF(COUNTIF('Lookup Net Position'!$B$2:$B$514,B16)=0,"acfr:CurrentAssetsCustom",_xlfn.XLOOKUP(B16,'Lookup Net Position'!$B$2:$B$514,'Lookup Net Position'!$C$2:$C$514)))</f>
         <v>Choose from drop-down --&gt;</v>
       </c>
-      <c r="B16" s="251"/>
+      <c r="B16" s="246"/>
       <c r="C16" s="202"/>
       <c r="D16" s="203"/>
       <c r="E16" s="200" t="str">
@@ -49021,17 +49013,17 @@
       <c r="D102" s="37"/>
     </row>
     <row r="103" spans="1:6">
-      <c r="B103" s="256"/>
+      <c r="B103" s="251"/>
     </row>
     <row r="104" spans="1:6">
-      <c r="A104" s="257"/>
-      <c r="B104" s="262" t="s">
+      <c r="A104" s="252"/>
+      <c r="B104" s="259" t="s">
         <v>3636</v>
       </c>
     </row>
     <row r="105" spans="1:6">
-      <c r="A105" s="257"/>
-      <c r="B105" s="263"/>
+      <c r="A105" s="252"/>
+      <c r="B105" s="260"/>
     </row>
   </sheetData>
   <sheetProtection formatRows="0" insertRows="0" deleteRows="0"/>
@@ -49320,20 +49312,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B9" s="15"/>
-      <c r="C9" s="242"/>
-      <c r="D9" s="243"/>
-      <c r="E9" s="243"/>
-      <c r="F9" s="243"/>
-      <c r="G9" s="244" t="str">
+      <c r="C9" s="202"/>
+      <c r="D9" s="203"/>
+      <c r="E9" s="203"/>
+      <c r="F9" s="203"/>
+      <c r="G9" s="226" t="str">
         <f>IF(OR(G$6="", B9=""),"",SUM(D9:F9) - C9)</f>
         <v/>
       </c>
-      <c r="H9" s="244"/>
-      <c r="I9" s="245" t="str">
+      <c r="H9" s="226"/>
+      <c r="I9" s="200" t="str">
         <f>IF(OR(I$6="", B9=""),"",SUM(G9:H9))</f>
         <v/>
       </c>
-      <c r="J9" s="244"/>
+      <c r="J9" s="226"/>
     </row>
     <row r="10" spans="1:10" ht="16">
       <c r="A10" s="50" t="str">
@@ -49341,20 +49333,17 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B10" s="15"/>
-      <c r="C10" s="242"/>
-      <c r="D10" s="243"/>
-      <c r="E10" s="243"/>
-      <c r="F10" s="243"/>
-      <c r="G10" s="244" t="str">
-        <f t="shared" ref="G10:G22" si="0">IF(OR(G$6="", B10=""),"",SUM(D10:F10) - C10)</f>
+      <c r="C10" s="202"/>
+      <c r="D10" s="203"/>
+      <c r="E10" s="203"/>
+      <c r="F10" s="203"/>
+      <c r="G10" s="226"/>
+      <c r="H10" s="226"/>
+      <c r="I10" s="200" t="str">
+        <f t="shared" ref="I10:I22" si="0">IF(OR(I$6="", B10=""),"",SUM(G10:H10))</f>
         <v/>
       </c>
-      <c r="H10" s="244"/>
-      <c r="I10" s="245" t="str">
-        <f t="shared" ref="I10:I22" si="1">IF(OR(I$6="", B10=""),"",SUM(G10:H10))</f>
-        <v/>
-      </c>
-      <c r="J10" s="244"/>
+      <c r="J10" s="226"/>
     </row>
     <row r="11" spans="1:10" ht="16">
       <c r="A11" s="50" t="str">
@@ -49362,20 +49351,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B11" s="15"/>
-      <c r="C11" s="242"/>
-      <c r="D11" s="243"/>
-      <c r="E11" s="243"/>
-      <c r="F11" s="243"/>
-      <c r="G11" s="244" t="str">
+      <c r="C11" s="202"/>
+      <c r="D11" s="203"/>
+      <c r="E11" s="203"/>
+      <c r="F11" s="203"/>
+      <c r="G11" s="226" t="str">
+        <f t="shared" ref="G10:G22" si="1">IF(OR(G$6="", B11=""),"",SUM(D11:F11) - C11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="226"/>
+      <c r="I11" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H11" s="244"/>
-      <c r="I11" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J11" s="244"/>
+      <c r="J11" s="226"/>
     </row>
     <row r="12" spans="1:10" ht="16">
       <c r="A12" s="50" t="str">
@@ -49383,20 +49372,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B12" s="15"/>
-      <c r="C12" s="242"/>
-      <c r="D12" s="243"/>
-      <c r="E12" s="243"/>
-      <c r="F12" s="243"/>
-      <c r="G12" s="244" t="str">
+      <c r="C12" s="202"/>
+      <c r="D12" s="203"/>
+      <c r="E12" s="203"/>
+      <c r="F12" s="203"/>
+      <c r="G12" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H12" s="226"/>
+      <c r="I12" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H12" s="244"/>
-      <c r="I12" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J12" s="244"/>
+      <c r="J12" s="226"/>
     </row>
     <row r="13" spans="1:10" ht="16">
       <c r="A13" s="50" t="str">
@@ -49404,20 +49393,17 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B13" s="15"/>
-      <c r="C13" s="242"/>
-      <c r="D13" s="243"/>
-      <c r="E13" s="243"/>
-      <c r="F13" s="243"/>
-      <c r="G13" s="244" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H13" s="244"/>
-      <c r="I13" s="245" t="str">
+      <c r="C13" s="202"/>
+      <c r="D13" s="203"/>
+      <c r="E13" s="203"/>
+      <c r="F13" s="203"/>
+      <c r="G13" s="226" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J13" s="244"/>
+      <c r="H13" s="226"/>
+      <c r="I13" s="200"/>
+      <c r="J13" s="226"/>
     </row>
     <row r="14" spans="1:10" ht="16">
       <c r="A14" s="50" t="str">
@@ -49425,20 +49411,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B14" s="15"/>
-      <c r="C14" s="242"/>
-      <c r="D14" s="243"/>
-      <c r="E14" s="243"/>
-      <c r="F14" s="243"/>
-      <c r="G14" s="244" t="str">
+      <c r="C14" s="202"/>
+      <c r="D14" s="203"/>
+      <c r="E14" s="203"/>
+      <c r="F14" s="203"/>
+      <c r="G14" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H14" s="226"/>
+      <c r="I14" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H14" s="244"/>
-      <c r="I14" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J14" s="244"/>
+      <c r="J14" s="226"/>
     </row>
     <row r="15" spans="1:10" ht="16">
       <c r="A15" s="50" t="str">
@@ -49446,20 +49432,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B15" s="15"/>
-      <c r="C15" s="242"/>
-      <c r="D15" s="243"/>
-      <c r="E15" s="243"/>
-      <c r="F15" s="243"/>
-      <c r="G15" s="244" t="str">
+      <c r="C15" s="202"/>
+      <c r="D15" s="203"/>
+      <c r="E15" s="203"/>
+      <c r="F15" s="203"/>
+      <c r="G15" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H15" s="226"/>
+      <c r="I15" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H15" s="244"/>
-      <c r="I15" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J15" s="244"/>
+      <c r="J15" s="226"/>
     </row>
     <row r="16" spans="1:10" ht="16">
       <c r="A16" s="50" t="str">
@@ -49467,20 +49453,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B16" s="15"/>
-      <c r="C16" s="242"/>
-      <c r="D16" s="243"/>
-      <c r="E16" s="243"/>
-      <c r="F16" s="243"/>
-      <c r="G16" s="244" t="str">
+      <c r="C16" s="202"/>
+      <c r="D16" s="203"/>
+      <c r="E16" s="203"/>
+      <c r="F16" s="203"/>
+      <c r="G16" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H16" s="226"/>
+      <c r="I16" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H16" s="244"/>
-      <c r="I16" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J16" s="244"/>
+      <c r="J16" s="226"/>
     </row>
     <row r="17" spans="1:10" ht="16">
       <c r="A17" s="50" t="str">
@@ -49488,20 +49474,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B17" s="15"/>
-      <c r="C17" s="242"/>
-      <c r="D17" s="243"/>
-      <c r="E17" s="243"/>
-      <c r="F17" s="243"/>
-      <c r="G17" s="244" t="str">
+      <c r="C17" s="202"/>
+      <c r="D17" s="203"/>
+      <c r="E17" s="203"/>
+      <c r="F17" s="203"/>
+      <c r="G17" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H17" s="226"/>
+      <c r="I17" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H17" s="244"/>
-      <c r="I17" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J17" s="244"/>
+      <c r="J17" s="226"/>
     </row>
     <row r="18" spans="1:10" ht="16" hidden="1">
       <c r="A18" s="50" t="str">
@@ -49509,20 +49495,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B18" s="15"/>
-      <c r="C18" s="242"/>
-      <c r="D18" s="243"/>
-      <c r="E18" s="243"/>
-      <c r="F18" s="243"/>
-      <c r="G18" s="244" t="str">
+      <c r="C18" s="202"/>
+      <c r="D18" s="203"/>
+      <c r="E18" s="203"/>
+      <c r="F18" s="203"/>
+      <c r="G18" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H18" s="226"/>
+      <c r="I18" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H18" s="244"/>
-      <c r="I18" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J18" s="244"/>
+      <c r="J18" s="226"/>
     </row>
     <row r="19" spans="1:10" ht="16" hidden="1">
       <c r="A19" s="50" t="str">
@@ -49530,20 +49516,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B19" s="15"/>
-      <c r="C19" s="242"/>
-      <c r="D19" s="243"/>
-      <c r="E19" s="243"/>
-      <c r="F19" s="243"/>
-      <c r="G19" s="244" t="str">
+      <c r="C19" s="202"/>
+      <c r="D19" s="203"/>
+      <c r="E19" s="203"/>
+      <c r="F19" s="203"/>
+      <c r="G19" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H19" s="226"/>
+      <c r="I19" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H19" s="244"/>
-      <c r="I19" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J19" s="244"/>
+      <c r="J19" s="226"/>
     </row>
     <row r="20" spans="1:10" ht="16" hidden="1">
       <c r="A20" s="50" t="str">
@@ -49551,20 +49537,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B20" s="15"/>
-      <c r="C20" s="242"/>
-      <c r="D20" s="243"/>
-      <c r="E20" s="243"/>
-      <c r="F20" s="243"/>
-      <c r="G20" s="244" t="str">
+      <c r="C20" s="202"/>
+      <c r="D20" s="203"/>
+      <c r="E20" s="203"/>
+      <c r="F20" s="203"/>
+      <c r="G20" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H20" s="226"/>
+      <c r="I20" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H20" s="244"/>
-      <c r="I20" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J20" s="244"/>
+      <c r="J20" s="226"/>
     </row>
     <row r="21" spans="1:10" ht="16" hidden="1">
       <c r="A21" s="50" t="str">
@@ -49572,20 +49558,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B21" s="15"/>
-      <c r="C21" s="242"/>
-      <c r="D21" s="243"/>
-      <c r="E21" s="243"/>
-      <c r="F21" s="243"/>
-      <c r="G21" s="244" t="str">
+      <c r="C21" s="202"/>
+      <c r="D21" s="203"/>
+      <c r="E21" s="203"/>
+      <c r="F21" s="203"/>
+      <c r="G21" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H21" s="226"/>
+      <c r="I21" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H21" s="244"/>
-      <c r="I21" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J21" s="244"/>
+      <c r="J21" s="226"/>
     </row>
     <row r="22" spans="1:10" ht="16">
       <c r="A22" s="50" t="str">
@@ -49593,20 +49579,20 @@
         <v>Choose from drop-down --&gt;</v>
       </c>
       <c r="B22" s="15"/>
-      <c r="C22" s="242"/>
-      <c r="D22" s="243"/>
-      <c r="E22" s="243"/>
-      <c r="F22" s="243"/>
-      <c r="G22" s="244" t="str">
+      <c r="C22" s="202"/>
+      <c r="D22" s="203"/>
+      <c r="E22" s="203"/>
+      <c r="F22" s="203"/>
+      <c r="G22" s="226" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H22" s="226"/>
+      <c r="I22" s="200" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H22" s="244"/>
-      <c r="I22" s="245" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J22" s="244"/>
+      <c r="J22" s="226"/>
     </row>
     <row r="23" spans="1:10" ht="15">
       <c r="A23" s="6" t="s">
@@ -49615,32 +49601,35 @@
       <c r="B23" s="6" t="s">
         <v>1100</v>
       </c>
-      <c r="C23" s="245">
-        <f t="shared" ref="C23:I23" si="2">IF(C6="","",SUM(C9:C22))</f>
-        <v>0</v>
-      </c>
-      <c r="D23" s="245">
+      <c r="C23" s="200"/>
+      <c r="D23" s="200">
+        <f t="shared" ref="C23:J23" si="2">IF(D6="","",SUM(D9:D22))</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="200">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E23" s="245">
+      <c r="F23" s="200">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F23" s="245">
+      <c r="G23" s="200">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G23" s="245">
+      <c r="H23" s="200">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="H23" s="245"/>
-      <c r="I23" s="245">
+      <c r="I23" s="200">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J23" s="245"/>
+      <c r="J23" s="200">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" spans="1:10" ht="15">
       <c r="A24" s="5"/>
@@ -49725,10 +49714,7 @@
       <c r="E28" s="203"/>
       <c r="F28" s="203"/>
       <c r="G28" s="226"/>
-      <c r="H28" s="226" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
+      <c r="H28" s="226"/>
       <c r="I28" s="200" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -49932,7 +49918,10 @@
         <f>IF(I$6="","",SUM(I25:I36))</f>
         <v>0</v>
       </c>
-      <c r="J37" s="200"/>
+      <c r="J37" s="200">
+        <f>IF(J$6="","",SUM(J25:J36))</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="38" spans="1:10" ht="15">
       <c r="A38" s="6" t="s">
@@ -49962,14 +49951,17 @@
         <v>0</v>
       </c>
       <c r="H38" s="204">
-        <f t="shared" ref="H38:I38" si="9">IF(H$6="","",H23+H37)</f>
+        <f t="shared" ref="H38:J38" si="9">IF(H$6="","",H23+H37)</f>
         <v>0</v>
       </c>
       <c r="I38" s="204">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J38" s="204"/>
+      <c r="J38" s="204">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="39" spans="1:10" ht="15">
       <c r="A39" s="5"/>
@@ -50029,12 +50021,9 @@
       <c r="D42" s="203"/>
       <c r="E42" s="203"/>
       <c r="F42" s="203"/>
-      <c r="G42" s="226" t="str">
-        <f t="shared" ref="G42:H49" si="11">IF(OR(G$6="", B42=""),"",0)</f>
-        <v/>
-      </c>
+      <c r="G42" s="226"/>
       <c r="H42" s="226" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="G42:H49" si="11">IF(OR(H$6="", C42=""),"",0)</f>
         <v/>
       </c>
       <c r="I42" s="200" t="str">
@@ -50056,10 +50045,7 @@
       <c r="D43" s="203"/>
       <c r="E43" s="203"/>
       <c r="F43" s="203"/>
-      <c r="G43" s="226" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
+      <c r="G43" s="226"/>
       <c r="H43" s="226" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -50083,10 +50069,7 @@
       <c r="D44" s="203"/>
       <c r="E44" s="203"/>
       <c r="F44" s="203"/>
-      <c r="G44" s="226" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
+      <c r="G44" s="226"/>
       <c r="H44" s="226" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -50110,10 +50093,7 @@
       <c r="D45" s="203"/>
       <c r="E45" s="203"/>
       <c r="F45" s="203"/>
-      <c r="G45" s="226" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
+      <c r="G45" s="226"/>
       <c r="H45" s="226" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -50627,7 +50607,10 @@
         <f>IF($C$6="","",SUM(G64:G70))</f>
         <v>0</v>
       </c>
-      <c r="H71" s="200"/>
+      <c r="H71" s="200">
+        <f>IF($C$6="","",SUM(H64:H70))</f>
+        <v>0</v>
+      </c>
       <c r="I71" s="200">
         <f>IF(I$6="","",SUM(I64:I70))</f>
         <v>0</v>
@@ -50690,16 +50673,16 @@
       <c r="D75" s="74"/>
       <c r="E75" s="74"/>
       <c r="F75" s="74"/>
-      <c r="G75" s="246">
+      <c r="G75" s="241">
         <f>G72+G23</f>
         <v>0</v>
       </c>
-      <c r="H75" s="246"/>
+      <c r="H75" s="241"/>
       <c r="I75" s="200">
         <f>IF(I$6="","",SUM(G75:H75))</f>
         <v>0</v>
       </c>
-      <c r="J75" s="246">
+      <c r="J75" s="241">
         <f>J72+J50</f>
         <v>0</v>
       </c>
@@ -50734,19 +50717,19 @@
       <c r="D77" s="74"/>
       <c r="E77" s="74"/>
       <c r="F77" s="74"/>
-      <c r="G77" s="247">
+      <c r="G77" s="242">
         <f>G75+G76</f>
         <v>0</v>
       </c>
-      <c r="H77" s="247">
+      <c r="H77" s="242">
         <f t="shared" ref="H77:J77" si="21">H75+H76</f>
         <v>0</v>
       </c>
-      <c r="I77" s="247">
+      <c r="I77" s="242">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="J77" s="247">
+      <c r="J77" s="242">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
@@ -50758,15 +50741,15 @@
       <c r="I79" s="54"/>
     </row>
     <row r="80" spans="1:10" ht="15">
-      <c r="A80" s="257"/>
-      <c r="B80" s="264" t="s">
+      <c r="A80" s="252"/>
+      <c r="B80" s="261" t="s">
         <v>3636</v>
       </c>
       <c r="I80" s="54"/>
     </row>
     <row r="81" spans="1:9" ht="15">
-      <c r="A81" s="257"/>
-      <c r="B81" s="265"/>
+      <c r="A81" s="252"/>
+      <c r="B81" s="262"/>
       <c r="I81" s="54"/>
     </row>
     <row r="82" spans="1:9" ht="15">
@@ -50893,12 +50876,12 @@
       <formula>H$6=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H38:I38">
+  <conditionalFormatting sqref="H38:J38">
     <cfRule type="expression" dxfId="66" priority="52" stopIfTrue="1">
       <formula>H$6=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:J6 D7:I37 I39:I51">
+  <conditionalFormatting sqref="H5:J6 I39:I51 D7:I37 J23 J37">
     <cfRule type="expression" dxfId="65" priority="48" stopIfTrue="1">
       <formula>D$6=""</formula>
     </cfRule>
@@ -50908,7 +50891,7 @@
       <formula>H$6=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J50">
+  <conditionalFormatting sqref="J7:J22 J24:J36 J39:J50">
     <cfRule type="expression" dxfId="63" priority="13" stopIfTrue="1">
       <formula>J$6=""</formula>
     </cfRule>

</xml_diff>